<commit_message>
fix(excel-workbook): correct README swap steps and percentile labels
Document the blank-row guard on Outputs, 1-based column constants, and
that outputs in .pd4castrrc.json must match OUTPUT_COLUMNS. Fix the
revenue sign claim for negative prices, label the percentile cells as
PERCENTILE arguments, and take the sheet name from OUTPUTS_SHEET in the
extra-rows error.
</commit_message>
<xml_diff>
--- a/examples/excel-workbook/model/battery_plan.xlsx
+++ b/examples/excel-workbook/model/battery_plan.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calc" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outputs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Calc" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Outputs" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -523,7 +523,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>fraction of the price range, 0 to 1</t>
+          <t>PERCENTILE of the prices, 0 to 1</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>fraction of the price range, 0 to 1</t>
+          <t>PERCENTILE of the prices, 0 to 1</t>
         </is>
       </c>
     </row>

</xml_diff>